<commit_message>
Explain why show rate can read above 100% on a one-week view
The audit of the converted sheets surfaced Show Rate at 100% and 125% in
the This Week and Last Week columns. That is real, not a formula fault: a
call booked on Friday is shown on Monday, so inside a fixed seven-day
window the shows can outnumber that window's bookings. It settles over
the month and all-time columns.

It will do this with real client data too, and a client seeing 125% would
reasonably conclude the sheet is broken, so the Cheat Sheet now says so
under Show rate — the place someone goes when a number looks wrong — and
tells them to judge show rate on the month, never on one week.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ByBdvAsLbjH7ye5fUDygK8
</commit_message>
<xml_diff>
--- a/docs/The_Called_Scoreboard.xlsx
+++ b/docs/The_Called_Scoreboard.xlsx
@@ -23485,7 +23485,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="17" customHeight="1">
+    <row r="41" ht="43" customHeight="1">
       <c r="A41" s="94" t="inlineStr">
         <is>
           <t>If it's high</t>
@@ -23493,7 +23493,7 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Your bookings are real. Push volume upstream.</t>
+          <t>Your bookings are real. Push volume upstream. Over a single week this can read above 100% — a call booked on Friday gets shown on Monday, so inside a 7-day window the shows can outnumber the bookings. It is not a broken number. Judge show rate on the month or all-time column, never on one week.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use The Called's own healthy ranges, not placeholder benchmarks
Francis set these directly in the live sheet: reply 50-80%, pitch 25-40%,
book 60-80%, show 70-90%, close 40-70%. They replace the working numbers
the build shipped with, which were mine and were only ever a stand-in.

Moving them into the content module means every future rebuild and the
Notion cheat sheet carry them, instead of the live sheet and the source
drifting apart the first time anyone regenerates.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ByBdvAsLbjH7ye5fUDygK8
</commit_message>
<xml_diff>
--- a/docs/The_Called_Scoreboard.xlsx
+++ b/docs/The_Called_Scoreboard.xlsx
@@ -23185,10 +23185,10 @@
         </is>
       </c>
       <c r="C11" s="89" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D11" s="89" t="n">
-        <v>0.25</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -23203,10 +23203,10 @@
         </is>
       </c>
       <c r="C12" s="89" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="D12" s="89" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -23221,10 +23221,10 @@
         </is>
       </c>
       <c r="C13" s="89" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="D13" s="89" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -23239,10 +23239,10 @@
         </is>
       </c>
       <c r="C14" s="89" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="D14" s="89" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -23257,10 +23257,10 @@
         </is>
       </c>
       <c r="C15" s="89" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D15" s="89" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">

</xml_diff>